<commit_message>
TD-7678 Update bulk relations creation to support concept type filtering, fix duplicate detection to preserve first occurrence, and normalize link_type and concept_type values
</commit_message>
<xml_diff>
--- a/test/fixtures/bulk_relations_empty_test.xlsx
+++ b/test/fixtures/bulk_relations_empty_test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bluetab/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzo.sanchez/workspace/truedat/back/td-lm/test/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F501CE-A45E-0940-B622-86E0983F54AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180F42BB-695B-1443-81DF-1B397BBA6B3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45000" yWindow="9420" windowWidth="18200" windowHeight="8500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="24000" windowHeight="36140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>concept_name</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>foo_domain</t>
+  </si>
+  <si>
+    <t>concept_type</t>
   </si>
 </sst>
 </file>
@@ -398,18 +401,19 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32.1640625" customWidth="1"/>
-    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.1640625" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -420,32 +424,35 @@
         <v>0</v>
       </c>
       <c r="D1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D2" t="s">
+    <row r="2" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>